<commit_message>
EMP -> Z (no rotate-camera clash); key hints read the live binding; no pan in Aster sim
- Rebind the emp action V->Z (project.godot + abilities.xlsx) so it no longer
  collides with E/rotate-camera. The old state showed [E] but fired on V.
- Add InputHints.label_for_action/bracket: derive prompt + HUD key labels from
  the actual InputMap binding (controller-aware, mobile-noted), never a baked
  letter. Wire the elevator EMP/pause prompts and the EMP ability hint through it.
- Aster sim camera: free_look off (small room) — follow + rotate + zoom stay,
  panning is disabled.
- Elevator tests now assert the prompt shows the LIVE emp key and press the bound
  key, so a future rebind can't desync them.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/abilities/en/abilities.xlsx
+++ b/to-rust-as-we-fall/data/abilities/en/abilities.xlsx
@@ -748,10 +748,6 @@
           <t>EMP</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1148,10 +1144,6 @@
           <t>PROTECT</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1560,8 +1552,6 @@
           <t>attacking</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1599,7 +1589,6 @@
           <t>18.0</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1632,7 +1621,6 @@
           <t>resting</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>12.0</t>
@@ -1660,10 +1648,6 @@
           <t>0.8,0.55,0.2</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1678,7 +1662,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1686,10 +1670,6 @@
           <t>0.29,0.62,1.0</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
rename "ferrolure" -> "flure" everywhere (one consistent term)
Project-wide rename of the lure mechanic from ferrolure to flure: code
identifiers, chunk ids, dialogue keys, ability keys, test flags/names, level &
puzzle docs, and the showcase fragment data. The mother_ferrolure chunk (script,
scene, board-layout doc, uid) is renamed to mother_flure; preview registries and
the --test-mother-flure flag follow. Dialogue (act1.xlsx) and ability
(abilities.xlsx) keys + text updated to match the renamed code references.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/abilities/en/abilities.xlsx
+++ b/to-rust-as-we-fall/data/abilities/en/abilities.xlsx
@@ -944,7 +944,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>mother_ferrolure.aster_focus</t>
+          <t>mother_flure.aster_focus</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -976,7 +976,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>mother_ferrolure.endo_patch</t>
+          <t>mother_flure.endo_patch</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1008,7 +1008,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>mother_ferrolure.peris_tune</t>
+          <t>mother_flure.peris_tune</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">

</xml_diff>

<commit_message>
decorative invasive flora (4 cultivar species, yellow-only Peris HARVEST reveal on Y, runback decor pass) + anti-homeless architecture (SpikeStrip + SET_PIECES 21-24); --preview=hostile_streets
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/abilities/en/abilities.xlsx
+++ b/to-rust-as-we-fall/data/abilities/en/abilities.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1462,6 +1462,38 @@
       <c r="F34" t="inlineStr">
         <is>
           <t>BLOOM stretches the lure window if the team hesitates on the way into the slit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>data_fragment.peris_harvest</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HARVEST</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Just pretty. Nothing to take.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Ornamental growth reads yellow. Once read, it can be cleared.</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1671,6 +1703,28 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>peris_harvest</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>peris</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1.0,0.84,0.25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>